<commit_message>
Actualizacao da pagina Agencia e Soft Skills
</commit_message>
<xml_diff>
--- a/Presencas_colectivas.xlsx
+++ b/Presencas_colectivas.xlsx
@@ -32297,13 +32297,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60A720EA-C7C5-4DDE-BFC2-39FB21775EAA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA135AA9-95D7-4942-8CE6-9C2401F550EF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7776E88-2C00-40B4-8D06-C7D53A0F830E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0EAFF2BF-15BB-4881-8B38-1375D0744DE0}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{308C8321-AF9D-4719-BB13-A7F2EDEE4898}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58B0C922-C4A0-42D6-9581-842CD94AC3FD}"/>
 </file>
</xml_diff>